<commit_message>
feat: implement live updates for course changes via Server-Sent Events
</commit_message>
<xml_diff>
--- a/docs/excel/api/CMAS-API-Endpoints.xlsx
+++ b/docs/excel/api/CMAS-API-Endpoints.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Security" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Endpoints'!$A$1:$R$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Endpoints'!$A$1:$R$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -986,7 +986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R78"/>
+  <dimension ref="A1:R79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7455,8 +7455,90 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="17" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="18" t="inlineStr">
+        <is>
+          <t>9 แดชบอร์ด</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D79" s="19" t="inlineStr">
+        <is>
+          <t>/api/v1/events</t>
+        </is>
+      </c>
+      <c r="E79" s="18" t="inlineStr">
+        <is>
+          <t>แจ้งหน้าจออื่นเมื่อรายวิชาถูกแก้ (SSE) ให้โหลดใหม่เอง</t>
+        </is>
+      </c>
+      <c r="F79" s="18" t="inlineStr">
+        <is>
+          <t>ผู้ใช้ที่ล็อกอิน</t>
+        </is>
+      </c>
+      <c r="G79" s="17" t="inlineStr">
+        <is>
+          <t>กรองในตัว</t>
+        </is>
+      </c>
+      <c r="H79" s="18" t="inlineStr">
+        <is>
+          <t>อ่าน</t>
+        </is>
+      </c>
+      <c r="I79" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J79" s="6" t="inlineStr">
+        <is>
+          <t>ทำแล้ว</t>
+        </is>
+      </c>
+      <c r="K79" s="17" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="L79" s="17" t="inlineStr"/>
+      <c r="M79" s="17" t="inlineStr"/>
+      <c r="N79" s="18" t="inlineStr">
+        <is>
+          <t>ส่งเฉพาะ courseId</t>
+        </is>
+      </c>
+      <c r="O79" s="18" t="inlineStr">
+        <is>
+          <t>อ่านรายการ</t>
+        </is>
+      </c>
+      <c r="P79" s="18" t="inlineStr">
+        <is>
+          <t>อ่านอย่างเดียว</t>
+        </is>
+      </c>
+      <c r="Q79" s="18" t="inlineStr">
+        <is>
+          <t>ล็อกอินทั่วไป</t>
+        </is>
+      </c>
+      <c r="R79" s="6" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R78"/>
+  <autoFilter ref="A1:R79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8049,7 +8131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11397,7 +11479,7 @@
     </row>
     <row r="75" ht="96" customHeight="1">
       <c r="A75" s="17" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
@@ -11406,12 +11488,12 @@
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>/api/v1/courses/:courseId/dashboard/attainment</t>
+          <t>/api/v1/events</t>
         </is>
       </c>
       <c r="D75" s="18" t="inlineStr">
         <is>
-          <t>:courseId</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E75" s="18" t="inlineStr">
@@ -11421,28 +11503,28 @@
       </c>
       <c r="F75" s="18" t="inlineStr">
         <is>
-          <t>200 · {classTarget, cloPassMark, helpCount, clos[{cloId, number, description, attainment, status, passedCount, evaluableCount, notEvaluatedCount, provisionalCount}]} · meta {computable, blockers[]}</t>
+          <t>200 · text/event-stream · ทุกครั้งที่เขียนสำเร็จ: data: {courseId, origin?} · ping ทุก 25 วินาที · server ปิด stream ทุก 10 นาที</t>
         </is>
       </c>
       <c r="G75" s="18" t="inlineStr">
         <is>
-          <t>401 · 404</t>
+          <t>401</t>
         </is>
       </c>
       <c r="H75" s="18" t="inlineStr">
         <is>
-          <t>ข้อมูลไม่พอ → attainment = null + blockers ห้ามส่ง 0 (FR-84) · helpCount = คนที่ยังไม่ผ่านอย่างน้อย 1 CLO</t>
+          <t>ส่งเฉพาะ courseId ให้ผู้สอนของวิชานั้นและ ADMIN (A-13) · ข้อมูลจริงยังอ่านผ่าน GET ที่ตรวจสิทธิ์ · token ส่งใน header ไม่ใช่ URL · origin คือ X-Client-Id ของแท็บที่เขียน</t>
         </is>
       </c>
       <c r="I75" s="18" t="inlineStr">
         <is>
-          <t>ST-CALC-01, 03</t>
+          <t>ST-ACL-06</t>
         </is>
       </c>
     </row>
     <row r="76" ht="96" customHeight="1">
       <c r="A76" s="7" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
@@ -11451,7 +11533,7 @@
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>/api/v1/courses/:courseId/dashboard/at-risk</t>
+          <t>/api/v1/courses/:courseId/dashboard/attainment</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
@@ -11466,7 +11548,7 @@
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>200 · [{studentId, studentCode, name, level (COURSE_FAIL|CLO_BELOW|OVERDUE), failedClos[{cloId, number, score, gap, near, provisional, hasPlan}], overdue[], totalScore, coursePassed}] · meta {atRiskCount, notEvaluatedCount, evaluatedCount}</t>
+          <t>200 · {classTarget, cloPassMark, helpCount, clos[{cloId, number, description, attainment, status, passedCount, evaluableCount, notEvaluatedCount, provisionalCount}]} · meta {computable, blockers[]}</t>
         </is>
       </c>
       <c r="G76" s="8" t="inlineStr">
@@ -11476,18 +11558,18 @@
       </c>
       <c r="H76" s="8" t="inlineStr">
         <is>
-          <t>ยังไม่มีคะแนนเลย ≠ at-risk (CR-03.1) · near = ห่างจากเกณฑ์ไม่เกิน 10 คะแนน (NEAR_GAP) · hasPlan บอกว่ามีแผนพัฒนาแล้ว</t>
+          <t>ข้อมูลไม่พอ → attainment = null + blockers ห้ามส่ง 0 (FR-84) · helpCount = คนที่ยังไม่ผ่านอย่างน้อย 1 CLO</t>
         </is>
       </c>
       <c r="I76" s="8" t="inlineStr">
         <is>
-          <t>ST-CALC-02</t>
+          <t>ST-CALC-01, 03</t>
         </is>
       </c>
     </row>
     <row r="77" ht="96" customHeight="1">
       <c r="A77" s="17" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
@@ -11496,12 +11578,12 @@
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>/api/v1/courses/:courseId/dashboard/students/:studentId</t>
+          <t>/api/v1/courses/:courseId/dashboard/at-risk</t>
         </is>
       </c>
       <c r="D77" s="18" t="inlineStr">
         <is>
-          <t>:courseId, :studentId</t>
+          <t>:courseId</t>
         </is>
       </c>
       <c r="E77" s="18" t="inlineStr">
@@ -11511,74 +11593,119 @@
       </c>
       <c r="F77" s="18" t="inlineStr">
         <is>
-          <t>200 · {student, gradeScale, clos[{cloId, number, score, passMark, status, objectives[]}], activities[], totalScore, coursePassed, passFailResult, remediationPlans[{cloId, plan, updatedAt}]}</t>
+          <t>200 · [{studentId, studentCode, name, level (COURSE_FAIL|CLO_BELOW|OVERDUE), failedClos[{cloId, number, score, gap, near, provisional, hasPlan}], overdue[], totalScore, coursePassed}] · meta {atRiskCount, notEvaluatedCount, evaluatedCount}</t>
         </is>
       </c>
       <c r="G77" s="18" t="inlineStr">
         <is>
-          <t>401 · 404 นักศึกษาไม่ใช่ของวิชานี้</t>
+          <t>401 · 404</t>
         </is>
       </c>
       <c r="H77" s="18" t="inlineStr">
         <is>
-          <t>PASS_FAIL ไม่ส่งเกรดตัวอักษร (CR-06) · คะแนนดิบอยู่คู่กับ % เสมอ (M5)</t>
+          <t>ยังไม่มีคะแนนเลย ≠ at-risk (CR-03.1) · near = ห่างจากเกณฑ์ไม่เกิน 10 คะแนน (NEAR_GAP) · hasPlan บอกว่ามีแผนพัฒนาแล้ว</t>
         </is>
       </c>
       <c r="I77" s="18" t="inlineStr">
         <is>
-          <t>ST-CALC-01 · ST-GRADE-02</t>
+          <t>ST-CALC-02</t>
         </is>
       </c>
     </row>
     <row r="78" ht="96" customHeight="1">
       <c r="A78" s="7" t="n">
+        <v>76</v>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C78" s="15" t="inlineStr">
+        <is>
+          <t>/api/v1/courses/:courseId/dashboard/students/:studentId</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>:courseId, :studentId</t>
+        </is>
+      </c>
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>200 · {student, gradeScale, clos[{cloId, number, score, passMark, status, objectives[]}], activities[], totalScore, coursePassed, passFailResult, remediationPlans[{cloId, plan, updatedAt}]}</t>
+        </is>
+      </c>
+      <c r="G78" s="8" t="inlineStr">
+        <is>
+          <t>401 · 404 นักศึกษาไม่ใช่ของวิชานี้</t>
+        </is>
+      </c>
+      <c r="H78" s="8" t="inlineStr">
+        <is>
+          <t>PASS_FAIL ไม่ส่งเกรดตัวอักษร (CR-06) · คะแนนดิบอยู่คู่กับ % เสมอ (M5)</t>
+        </is>
+      </c>
+      <c r="I78" s="8" t="inlineStr">
+        <is>
+          <t>ST-CALC-01 · ST-GRADE-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="96" customHeight="1">
+      <c r="A79" s="17" t="n">
         <v>77</v>
       </c>
-      <c r="B78" s="6" t="inlineStr">
+      <c r="B79" s="6" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C78" s="15" t="inlineStr">
+      <c r="C79" s="19" t="inlineStr">
         <is>
           <t>/api/v1/courses/:courseId/dashboard/export</t>
         </is>
       </c>
-      <c r="D78" s="8" t="inlineStr">
+      <c r="D79" s="18" t="inlineStr">
         <is>
           <t>:courseId · scope=course|student, studentId?, format=xlsx</t>
         </is>
       </c>
-      <c r="E78" s="8" t="inlineStr">
+      <c r="E79" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F78" s="8" t="inlineStr">
+      <c r="F79" s="18" t="inlineStr">
         <is>
           <t>200 · xlsx</t>
         </is>
       </c>
-      <c r="G78" s="8" t="inlineStr">
+      <c r="G79" s="18" t="inlineStr">
         <is>
           <t>401 ไม่มี token · 400 scope=student แต่ไม่มี studentId · 403 ADMIN · 404</t>
         </is>
       </c>
-      <c r="H78" s="8" t="inlineStr">
+      <c r="H79" s="18" t="inlineStr">
         <is>
           <t>service เดียวกับ attainment / at-risk / รายงานรายบุคคล (FR-88) · S-7 · PDF หลัง v1</t>
         </is>
       </c>
-      <c r="I78" s="8" t="inlineStr">
+      <c r="I79" s="18" t="inlineStr">
         <is>
           <t>ST-CALC-04</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>ออกแบบครบ 77 จาก 77 endpoint · 4 ตัวเลื่อนไปหลัง v1 (D-5) ระบุไว้ว่าไม่ทำ · ตรวจกับระบบจริงด้วย scripts/check-api-design.py และ app/server/src/api-contract.test.ts</t>
+    <row r="81">
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>ออกแบบครบ 78 จาก 78 endpoint · 4 ตัวเลื่อนไปหลัง v1 (D-5) ระบุไว้ว่าไม่ทำ · ตรวจกับระบบจริงด้วย scripts/check-api-design.py และ app/server/src/api-contract.test.ts</t>
         </is>
       </c>
     </row>

</xml_diff>